<commit_message>
feat: vendor-search overhaul — offline per-category brand search + outputs
- New scripts/build_vendor_search.py: offline per-category vendor/brand search
  via the shared cve_search engine (description + CPE, whole_word) against the
  fixed NVD snapshot, mirroring build_keyword_search.py
- cve_search.py: add whole_word matching mode to filter_by_keywords
- build_keyword_search.py: use whole_word=True
- Add vendor_terms.csv / vendor_terms_proposed.csv / PROPOSED_brand_lists.md
- Rebuild all 14 existing results_all_*.xlsx on the snapshot; add 10 new
  category vendor lists; back up pre-rebuild files under
  _backup_pre_rebuild_2026-06-28/
- Add per-category keyword_*.csv outputs for all categories
</commit_message>
<xml_diff>
--- a/data/vendor-search/results_all_thermostat.xlsx
+++ b/data/vendor-search/results_all_thermostat.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,31 +481,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CVE-2001-0827</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>37231</v>
+          <t>CVE-2001-1295</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2001-08-21</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cerberus FTP server 1.0 - 1.5 allows remote attackers to cause a denial of service (crash) via a large number of "PASV" requests.</t>
+          <t>Directory traversal vulnerability in Cerberus FTP Server 1.5 and earlier allows remote attackers to read arbitrary files via a .. (dot dot) in the CD command.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CWE-400</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:grant_averett:ceberus_ftp_server:1.0:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.3:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.22:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:grant_averett:cerberus_ftp_server:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -517,11 +511,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>No</t>
@@ -540,8 +530,10 @@
           <t>CVE-2001-0702</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>37154</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2001-09-20</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -581,27 +573,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CVE-2001-1295</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>37124</v>
+          <t>CVE-2001-0827</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2001-12-06</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Directory traversal vulnerability in Cerberus FTP Server 1.5 and earlier allows remote attackers to read arbitrary files via a .. (dot dot) in the CD command.</t>
+          <t>Cerberus FTP server 1.0 - 1.5 allows remote attackers to cause a denial of service (crash) via a large number of "PASV" requests.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>3.1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CWE-400</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:grant_averett:cerberus_ftp_server:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:grant_averett:ceberus_ftp_server:1.0:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.3:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:grant_averett:ceberus_ftp_server:1.22:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -609,7 +607,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>No</t>
@@ -628,8 +630,10 @@
           <t>CVE-2003-1476</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>37986</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2003-12-31</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -669,31 +673,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CVE-2004-2769</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>40361</v>
+          <t>CVE-2005-1962</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2005-06-16</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cerberus FTP Server before 4.0.3.0 allows remote authenticated users to list hidden files, even when the "Display hidden files" option is enabled, via the (1) MLSD or (2) MLST commands.</t>
+          <t>Cross-site scripting (XSS) vulnerability in Cerberus Helpdesk 0.97.3 allows remote attackers to inject arbitrary web script or HTML via the (1) errorcode parameter to index.php or (2) certain fields to clients.php.</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>CWE-264</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -717,19 +719,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CVE-2005-4427</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>38706</v>
+          <t>CVE-2005-1963</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2005-06-16</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Multiple SQL injection vulnerabilities in Cerberus Helpdesk allow remote attackers to execute arbitrary SQL commands via the (1) file_id parameter to attachment_send.php, (2) the $addy variable in email_parser.php, (3) $address variable in email_parser.php, (4) $a_address variable in structs.php, (5) kbid parameter to cer_KnowledgebaseHandler.class.php, (6) queues[] parameter to addresses_export.php, (7) $thread variable to display.php, (8) ticket parameter to display_ticket_thread.php.</t>
+          <t>Cerberus Helpdesk 0.97.3 allows remote attackers to obtain sensitive information via certain requests to (1) reports.php, (2) knowledgebase.php, or (3) configuration.php, which leaks the information in a PHP error message.</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
@@ -737,7 +741,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.649:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -761,19 +765,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CVE-2005-4428</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>38706</v>
+          <t>CVE-2006-4539</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2006-09-05</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cross-site scripting (XSS) vulnerability in index.php in Cerberus Helpdesk allows remote attackers to inject arbitrary web script or HTML via the kb_ask parameter.</t>
+          <t>(1) includes/widgets/module_company_tickets.php and (2) includes/widgets/module_track_tickets.php Client Support Center in Cerberus Helpdesk 3.2 Build 317, and possibly earlier, allows remote attackers to bypass security restrictions and obtain sensitive information via the ticket parameter.  NOTE: the provenance of this information is unknown; the details are obtained from third party information.</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4.3</v>
+        <v>7.5</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
@@ -781,7 +787,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.649:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:3.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -805,27 +811,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CVE-2005-3502</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>38661</v>
+          <t>CVE-2007-5930</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2007-11-10</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>attachment_send.php in Cerberus Helpdesk allows remote attackers to view attachments and tickets of other users via a modified file_id parameter.</t>
+          <t>Cross-site scripting (XSS) vulnerability in the web interface in Cerberus FTP Server before 2.46 allows remote attackers to inject arbitrary web script or HTML via unspecified vectors.</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.6.1:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:ftp_server:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -849,27 +861,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CVE-2005-1962</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>38519</v>
+          <t>CVE-2004-2769</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2010-07-02</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cross-site scripting (XSS) vulnerability in Cerberus Helpdesk 0.97.3 allows remote attackers to inject arbitrary web script or HTML via the (1) errorcode parameter to index.php or (2) certain fields to clients.php.</t>
+          <t>Cerberus FTP Server before 4.0.3.0 allows remote authenticated users to list hidden files, even when the "Display hidden files" option is enabled, via the (1) MLSD or (2) MLST commands.</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CWE-264</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -893,19 +911,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CVE-2005-1963</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>38519</v>
+          <t>CVE-2014-8120</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2014-12-18</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cerberus Helpdesk 0.97.3 allows remote attackers to obtain sensitive information via certain requests to (1) reports.php, (2) knowledgebase.php, or (3) configuration.php, which leaks the information in a PHP error message.</t>
+          <t>The agent in Thermostat before 1.0.6, when using unspecified configurations, allows local users to obtain the JMX management URLs of all local Java virtual machines and gain privileges via unknown vectors.</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -913,12 +933,12 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:thermostat_project:thermostat:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -937,38 +957,44 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CVE-2006-6366</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>39058</v>
+          <t>CVE-2015-2867</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2017-01-06</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cross-site scripting (XSS) vulnerability in includes/elements/spellcheck/spellwin.php in Cerberus Helpdesk 0.97.3, 2.0 through 2.7, 3.2.1, and 3.3 allows remote attackers to inject arbitrary web script or HTML via the js parameter.  NOTE: The provenance of this information is unknown; the details are obtained solely from third party information.</t>
+          <t>A design flaw in the Trane ComfortLink II SCC firmware version 2.0.2 service allows remote attackers to take complete control of the system.</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CWE-798</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:helpdesk:0.97.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.6.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.2.317:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.3:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -981,38 +1007,44 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CVE-2006-5428</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>39010</v>
+          <t>CVE-2015-2868</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2017-01-06</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>rpc.php in Cerberus Helpdesk 3.2.1 does not verify a client's privileges for a display_get_requesters operation, which allows remote attackers to bypass the GUI login and obtain sensitive information (ticket data) via a direct request.</t>
+          <t>An exploitable remote code execution vulnerability exists in the Trane ComfortLink II firmware version 2.0.2 in DSS service. An attacker who can connect to the DSS service on the Trane ComfortLink II device can send an overly long REG request that can overflow a fixed size stack buffer, resulting in arbitrary code execution.</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CWE-119</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:3.2.1:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -1025,71 +1057,71 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CVE-2006-4539</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>38965</v>
+          <t>CVE-2014-8362</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2017-01-23</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>(1) includes/widgets/module_company_tickets.php and (2) includes/widgets/module_track_tickets.php Client Support Center in Cerberus Helpdesk 3.2 Build 317, and possibly earlier, allows remote attackers to bypass security restrictions and obtain sensitive information via the ticket parameter.  NOTE: the provenance of this information is unknown; the details are obtained from third party information.</t>
+          <t>Vivint Sky Control Panel 1.1.1.9926 allows remote attackers to enable and disable the alarm system and modify other security settings via the Web-enabled interface.</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CWE-284</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:3.2:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:vivint:sky_control_panel_firmware:1.1.1.9926:*:*:*:*:*:*:*|cpe:2.3:h:vivint:sky_control_panel:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CVE-2006-0509</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>38749</v>
+          <t>CVE-2017-6367</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2017-03-14</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Multiple cross-site scripting (XSS) vulnerabilities in clients.php in Cerberus Helpdesk, possibly 2.7, allow remote attackers to inject arbitrary web script or HTML via (1) the contact_search parameter and (2) unspecified url fields.</t>
+          <t>In Cerberus FTP Server 8.0.10.1, a crafted HTTP request causes the Windows service to crash. The attack methodology involves a long Host header and an invalid Content-Length header.</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4.3</v>
+        <v>7.5</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CWE-20</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.7.1_development_release:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:8.0.10.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1113,27 +1145,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CVE-2006-0357</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>38739</v>
+          <t>CVE-2017-6880</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2017-03-17</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Grant Averett Cerberus FTP Server 2.32, and possibly earlier versions, allows remote attackers to cause an unspecified denial of service via a long string that does not contain a valid FTP command.</t>
+          <t>Buffer overflow in Cerberus FTP Server 8.0.10.3 allows remote attackers to cause a denial of service (daemon crash) or possibly have unspecified other impact via a long MLST command.</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CWE-119</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:grant_averett:cerberus_ftp_server:2.32:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_ftp_server:8.0.10.3:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1157,42 +1195,44 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CVE-2007-5930</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>39396</v>
+          <t>CVE-2018-11315</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2018-05-20</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cross-site scripting (XSS) vulnerability in the web interface in Cerberus FTP Server before 2.46 allows remote attackers to inject arbitrary web script or HTML via unspecified vectors.</t>
+          <t>The Local HTTP API in Radio Thermostat CT50 and CT80 1.04.84 and below products allows unauthorized access via a DNS rebinding attack. This can result in remote device temperature control, as demonstrated by a tstat t_heat request that accesses a device purchased in the Spring of 2018, and sets a home's target temperature to 95 degrees Fahrenheit. This vulnerability might be described as an addendum to CVE-2013-4860.</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4.3</v>
+        <v>6.5</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CWE-79</t>
+          <t>CWE-20</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:ftp_server:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:radiothermostat:ct50_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:radiothermostat:ct80_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct80:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1205,36 +1245,38 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CVE-2008-6440</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>39878</v>
+          <t>CVE-2018-14825</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2018-09-24</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cerberus Helpdesk before 4.0 (Build 600) allows remote attackers to obtain sensitive information via direct requests for "controllers ... that aren't standard helpdesk pages," possibly involving the (1) /display and (2) /kb URIs.</t>
+          <t>On Honeywell Mobile Computers (CT60 running Android OS 7.1, CN80 running Android OS 7.1, CT40 running Android OS 7.1, CK75 running Android OS 6.0, CN75 running Android OS 6.0, CN75e running Android OS 6.0, CT50 running Android OS 6.0, D75e running Android OS 6.0, CT50 running Android OS 4.4, D75e running Android OS 4.4, CN51 running Android OS 6.0, EDA50k running Android 4.4, EDA50 running Android OS 7.1, EDA50k running Android OS 7.1, EDA70 running Android OS 7.1, EDA60k running Android OS 7.1, and EDA51 running Android OS 8.1), a skilled attacker with advanced knowledge of the target system could exploit this vulnerability by creating an application that would successfully bind to the service and gain elevated system privileges. This could enable the attacker to obtain access to keystrokes, passwords, personal identifiable information, photos, emails, or business-critical documents.</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CWE-287</t>
+          <t>CWE-269|CWE-732</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:*:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.6.1:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.7.1:development_release:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.649:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:3.2:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:3.2.1:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:h:honeywell:cn80:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct40:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct60:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda50:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda50k:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda60k:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda70:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:7.1.0:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ck75:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn51:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn75:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn75e:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:d75e:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:6.0:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:4.4:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda51:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:8.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1253,127 +1295,109 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CVE-2008-3397</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>39660</v>
+          <t>CVE-2018-19588</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2019-07-11</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cross-site scripting (XSS) vulnerability in Runesoft Cerberus CMS before 3_1.4_0.9 allows remote attackers to inject arbitrary web script or HTML via a cerberus_user cookie.</t>
+          <t>Alarm.com ADC-V522IR 0100b9 devices have Incorrect Access Control.</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="E19" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CWE-79</t>
+          <t>CWE-284</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:runesoft:cerberus_cms:*:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:alarm:adc-v522ir_firmware:0100b9:*:*:*:*:*:*:*|cpe:2.3:h:alarm:adc-v522ir:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CVE-2012-6339</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>41274</v>
+          <t>CVE-2019-9657</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2019-07-11</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Multiple cross-site scripting (XSS) vulnerabilities in the administrative web interface in Cerberus FTP Server before 5.0.6.0 allow (1) remote attackers to inject arbitrary web script or HTML via a log entry that is not properly handled within the Log Manager component, and might allow (2) remote authenticated administrators to inject arbitrary web script or HTML via a Messages field to the servermanager program.</t>
+          <t>Alarm.com ADC-V522IR 0100b9 devices have Incorrect Access Control, a different issue than CVE-2018-19588. This occurs because of incorrect protection of VPN certificates (used for initiating a VPN session to the Alarm.com infrastructure) on the local camera device.</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4.3</v>
+        <v>7.8</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CWE-79</t>
+          <t>CWE-522</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.10.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.11.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.5.0:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:alarm:adc-v522ir_firmware:0100b9:*:*:*:*:*:*:*|cpe:2.3:h:alarm:adc-v522ir:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CVE-2012-2999</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>41186</v>
+          <t>CVE-2020-5195</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2020-01-13</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Multiple cross-site request forgery (CSRF) vulnerabilities in the web interface in Cerberus FTP Server before 5.0.5.0 allow remote attackers to hijack the authentication of administrators for requests that (1) add a user account or (2) reconfigure the state of the FTP service, as demonstrated by a request to usermanager/users/modify.</t>
+          <t>Reflected XSS through an IMG element in Cerberus FTP Server prior to versions 11.0.1 and 10.0.17 allows a remote attacker to execute arbitrary JavaScript or HTML via a crafted public folder URL. This occurs because of the folder_up.png IMG element not properly sanitizing user-inserted directory paths. The path modification must be done on a publicly shared folder for a remote attacker to insert arbitrary JavaScript or HTML. The vulnerability impacts anyone who clicks the malicious link crafted by the attacker.</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CWE-352</t>
+          <t>CWE-79</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.2:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1397,31 +1421,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CVE-2012-5301</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>41186</v>
+          <t>CVE-2020-5194</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2020-01-14</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>The default configuration of Cerberus FTP Server before 5.0.4.0 supports the DES cipher for SSH sessions, which makes it easier for remote attackers to obtain sensitive information by sniffing the network and performing a brute-force attack on the encrypted data.</t>
+          <t>The zip API endpoint in Cerberus FTP Server 8 allows an authenticated attacker without zip permission to use the zip functionality via an unrestricted API endpoint. Improper permission verification occurs when calling the file/ajax_download_zip/zip_name endpoint. The result is that a user without permissions can zip and download files even if they do not have permission to view whether the file exists.</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CWE-310</t>
+          <t>CWE-639</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.10.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.11.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:8.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1445,36 +1471,38 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CVE-2012-4006</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>41138</v>
+          <t>CVE-2020-5196</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2020-01-14</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The GREE application before 1.4.0, GREE Tanken Dorirando application before 1.0.7, GREE Tsurisuta application before 1.5.0, GREE Monpura application before 1.1.1, GREE Kaizokuoukoku Columbus application before 1.3.5, GREE haconiwa application before 1.1.0, GREE Seisen Cerberus application before 1.1.0, and KDDI&amp;GREE GREE Market application before 2.1.2 for Android do not properly implement the WebView class, which allows remote attackers to obtain sensitive information via a crafted application.</t>
+          <t>Cerberus FTP Server Enterprise Edition prior to versions 11.0.3 and 10.0.18 allows an authenticated attacker to create files, display hidden files, list directories, and list files without the permission to zip and download (or unzip and upload) files. There are multiple ways to bypass certain permissions by utilizing the zip and unzip features. As a result, users without permission can see files, folders, and hidden files, and can create directories without permission.</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.3</v>
+        <v>8.1</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CWE-200</t>
+          <t>CWE-276</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:gree:gree:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:haconiwa:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:kaizokuoukoku_columbus:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:monpura:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:seisen_cerberus:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:tanken_dorirando:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:tsurisuta:*:*:*:*:*:*:*:*|cpe:2.3:a:kddi_\&amp;_gree:gree_market:*:*:*:*:*:*:*:*|cpe:2.3:o:google:android:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1493,230 +1521,228 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CVE-2013-4860</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="n">
-        <v>41795</v>
+          <t>CVE-2021-37181</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2021-09-14</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Radio Thermostat CT80 And CT50 with firmware 1.4.64 and earlier does not restrict access to the API, which allows remote attackers to change the operation mode, wifi connection settings, temperature thresholds, and other settings via unspecified vectors.</t>
+          <t>A vulnerability has been identified in Cerberus DMS V4.0 (All versions), Cerberus DMS V4.1 (All versions), Cerberus DMS V4.2 (All versions), Cerberus DMS V5.0 (All versions &lt; v5.0 QU1), Desigo CC Compact V4.0 (All versions), Desigo CC Compact V4.1 (All versions), Desigo CC Compact V4.2 (All versions), Desigo CC Compact V5.0 (All versions &lt; V5.0 QU1), Desigo CC V4.0 (All versions), Desigo CC V4.1 (All versions), Desigo CC V4.2 (All versions), Desigo CC V5.0 (All versions &lt; V5.0 QU1). The application deserialises untrusted data without sufficient validations, that could result in an arbitrary deserialization. This could allow an unauthenticated attacker to execute code in the affected system. The CCOM communication component used for Windows App / Click-Once and IE Web / XBAP client connectivity are affected by the vulnerability.</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CWE-264</t>
+          <t>CWE-502</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:radiothermostat:ct50_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:radiothermostat:ct80_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct80:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:siemens:cerberus_dms:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:5.0:-:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:5.0:-:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:5.0:-:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Siemens Cerberus DMS and Desigo CC are enterprise building management/fire alarm platforms used in commercial buildings, not residential homes. Fails criterion 1 — not a residential deployment without dedicated security oversight.</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CVE-2014-8120</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="n">
-        <v>41991</v>
+          <t>CVE-2021-42534</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2021-10-22</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>The agent in Thermostat before 1.0.6, when using unspecified configurations, allows local users to obtain the JMX management URLs of all local Java virtual machines and gain privileges via unknown vectors.</t>
+          <t>The affected product’s web application does not properly neutralize the input during webpage generation, which could allow an attacker to inject code in the input forms.</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
+        <v>3.1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:thermostat_project:thermostat:*:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Maybe</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CVE-2015-2867</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>42741</v>
+          <t>CVE-2021-38450</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2021-10-27</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A design flaw in the Trane ComfortLink II SCC firmware version 2.0.2 service allows remote attackers to take complete control of the system.</t>
+          <t>The affected controllers do not properly sanitize the input containing code syntax. As a result, an attacker could craft code to alter the intended controller flow of the software.</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9.800000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CWE-798</t>
+          <t>CWE-94</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:5.5:-:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:-:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:5.5:-:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CVE-2015-2868</t>
-        </is>
-      </c>
-      <c r="B27" s="1" t="n">
-        <v>42741</v>
+          <t>CVE-2022-33139</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2022-06-21</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>An exploitable remote code execution vulnerability exists in the Trane ComfortLink II firmware version 2.0.2 in DSS service. An attacker who can connect to the DSS service on the Trane ComfortLink II device can send an overly long REG request that can overflow a fixed size stack buffer, resulting in arbitrary code execution.</t>
+          <t>A vulnerability has been identified in Cerberus DMS (All versions), Desigo CC (All versions), Desigo CC Compact (All versions), SIMATIC WinCC OA V3.16 (All versions in default configuration), SIMATIC WinCC OA V3.17 (All versions in non-default configuration), SIMATIC WinCC OA V3.18 (All versions in non-default configuration). Affected applications use client-side only authentication, when neither server-side authentication (SSA) nor Kerberos authentication is enabled. In this configuration, attackers could impersonate other users or exploit the client-server protocol without being authenticated.</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CWE-119</t>
+          <t>CWE-603|CWE-287</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:trane:comfortlink_ii_firmware:2.0.2:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:siemens:cerberus_dms:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.16:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.17:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.18:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Siemens Cerberus DMS and WinCC OA are industrial SCADA/building automation platforms. Same reasoning as CVE-2021-37181 — fails criterion 1 (residential deployment without dedicated security oversight).</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CVE-2015-3201</t>
-        </is>
-      </c>
-      <c r="B28" s="1" t="n">
-        <v>42163</v>
+          <t>CVE-2022-43704</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2023-01-20</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Thermostat before 2.0.0 uses world-readable permissions for the web.xml configuration file, which allows local users to obtain user credentials by reading the file.</t>
+          <t>The Sinilink XY-WFT1 WiFi Remote Thermostat, running firmware 1.3.6, allows an attacker to bypass the intended requirement to communicate using MQTT. It is possible to replay Sinilink aka SINILINK521 protocol (udp/1024) commands interfacing directly with the target device. This, in turn, allows for an attack to control the onboard relay without requiring authentication via the mobile application. This might result in an unacceptable temperature within the target device's physical environment.</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.1</v>
+        <v>5.9</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CWE-200</t>
+          <t>CWE-294</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:redhat:thermostat:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:sinilink:xy-wft1_firmware:1.3.6:*:*:*:*:*:*:*|cpe:2.3:h:sinilink:xy-wft1:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -1729,42 +1755,40 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CVE-2017-6880</t>
-        </is>
-      </c>
-      <c r="B29" s="1" t="n">
-        <v>42811</v>
+          <t>CVE-2023-24678</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2023-03-17</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Buffer overflow in Cerberus FTP Server 8.0.10.3 allows remote attackers to cause a denial of service (daemon crash) or possibly have unspecified other impact via a long MLST command.</t>
+          <t>A vulnerability in Centralite Pearl Thermostat 0x04075010 allows attackers to cause a Denial of Service (DoS) via a crafted Zigbee message.</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>CWE-119</t>
-        </is>
-      </c>
+        <v>3.1</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberus:cerberus_ftp_server:8.0.10.3:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:centralite:pearl_firmware:0x04075010:*:*:*:*:*:*:*|cpe:2.3:h:centralite:pearl:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -1777,31 +1801,29 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CVE-2017-6367</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>42808</v>
+          <t>CVE-2005-3502</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2005-11-05</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>In Cerberus FTP Server 8.0.10.1, a crafted HTTP request causes the Windows service to crash. The attack methodology involves a long Host header and an invalid Content-Length header.</t>
+          <t>attachment_send.php in Cerberus Helpdesk allows remote attackers to view attachments and tickets of other users via a modified file_id parameter.</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>CWE-20</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:8.0.10.1:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.6.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1825,42 +1847,40 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CVE-2018-6402</t>
-        </is>
-      </c>
-      <c r="B31" s="1" t="n">
-        <v>43935</v>
+          <t>CVE-2005-4427</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2005-12-20</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ecobee Ecobee4 4.2.0.171 devices can be forced to deauthenticate and connect to an unencrypted Wi-Fi network with the same SSID, even if the device settings specify use of encryption such as WPA2, as long as the competing network has a stronger signal. An attacker must be able to set up a nearby SSID, similar to an "Evil Twin" attack.</t>
+          <t>Multiple SQL injection vulnerabilities in Cerberus Helpdesk allow remote attackers to execute arbitrary SQL commands via the (1) file_id parameter to attachment_send.php, (2) the $addy variable in email_parser.php, (3) $address variable in email_parser.php, (4) $a_address variable in structs.php, (5) kbid parameter to cer_KnowledgebaseHandler.class.php, (6) queues[] parameter to addresses_export.php, (7) $thread variable to display.php, (8) ticket parameter to display_ticket_thread.php.</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>7.5</v>
       </c>
       <c r="E31" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>CWE-327</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:ecobee:ecobee4_firmware:4.2.0.171:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee4:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.649:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -1873,36 +1893,34 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CVE-2018-14825</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="n">
-        <v>43367</v>
+          <t>CVE-2005-4428</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2005-12-20</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>On Honeywell Mobile Computers (CT60 running Android OS 7.1, CN80 running Android OS 7.1, CT40 running Android OS 7.1, CK75 running Android OS 6.0, CN75 running Android OS 6.0, CN75e running Android OS 6.0, CT50 running Android OS 6.0, D75e running Android OS 6.0, CT50 running Android OS 4.4, D75e running Android OS 4.4, CN51 running Android OS 6.0, EDA50k running Android 4.4, EDA50 running Android OS 7.1, EDA50k running Android OS 7.1, EDA70 running Android OS 7.1, EDA60k running Android OS 7.1, and EDA51 running Android OS 8.1), a skilled attacker with advanced knowledge of the target system could exploit this vulnerability by creating an application that would successfully bind to the service and gain elevated system privileges. This could enable the attacker to obtain access to keystrokes, passwords, personal identifiable information, photos, emails, or business-critical documents.</t>
+          <t>Cross-site scripting (XSS) vulnerability in index.php in Cerberus Helpdesk allows remote attackers to inject arbitrary web script or HTML via the kb_ask parameter.</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5.8</v>
+        <v>4.3</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>CWE-269|CWE-732</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>cpe:2.3:h:honeywell:cn80:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct40:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct60:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda50:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda50k:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda60k:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda70:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:7.1.0:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ck75:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn51:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn75:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:cn75e:-:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:d75e:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:6.0:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:4.4:*:*:*:*:*:*:*|cpe:2.3:h:honeywell:eda51:-:*:*:*:*:*:*:*|cpe:2.3:o:google:android:8.1:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.649:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -1921,42 +1939,40 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CVE-2018-11315</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="n">
-        <v>43240</v>
+          <t>CVE-2006-0357</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2006-01-22</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>The Local HTTP API in Radio Thermostat CT50 and CT80 1.04.84 and below products allows unauthorized access via a DNS rebinding attack. This can result in remote device temperature control, as demonstrated by a tstat t_heat request that accesses a device purchased in the Spring of 2018, and sets a home's target temperature to 95 degrees Fahrenheit. This vulnerability might be described as an addendum to CVE-2013-4860.</t>
+          <t>Grant Averett Cerberus FTP Server 2.32, and possibly earlier versions, allows remote attackers to cause an unspecified denial of service via a long string that does not contain a valid FTP command.</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>CWE-20</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:radiothermostat:ct50_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:radiothermostat:ct80_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct80:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:grant_averett:cerberus_ftp_server:2.32:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -1969,31 +1985,29 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CVE-2019-25046</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="n">
-        <v>44357</v>
+          <t>CVE-2006-0509</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2006-02-01</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>The Web Client in Cerberus FTP Server Enterprise before 10.0.19 and 11.x before 11.0.4 allows XSS via an SVG document.</t>
+          <t>Multiple cross-site scripting (XSS) vulnerabilities in clients.php in Cerberus Helpdesk, possibly 2.7, allow remote attackers to inject arbitrary web script or HTML via (1) the contact_search parameter and (2) unspecified url fields.</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.1</v>
+        <v>4.3</v>
       </c>
       <c r="E34" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>CWE-79</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:cerberus_helpdesk:2.7.1_development_release:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2017,31 +2031,29 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CVE-2019-13466</t>
-        </is>
-      </c>
-      <c r="B35" s="1" t="n">
-        <v>43738</v>
+          <t>CVE-2006-5428</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2006-10-20</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Western Digital SSD Dashboard before 2.5.1.0 and SanDisk SSD Dashboard before 2.5.1.0 have Incorrect Access Control. The “generate reports” archive is protected with a hard-coded password. An application update that addresses the protection of archive encryption is available.</t>
+          <t>rpc.php in Cerberus Helpdesk 3.2.1 does not verify a client's privileges for a display_get_requesters operation, which allows remote attackers to bypass the GUI login and obtain sensitive information (ticket data) via a direct request.</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>CWE-798</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:sandisk:ssd_dashboard:*:*:*:*:*:*:*:*|cpe:2.3:a:westerndigital:ssd_dashboard:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:3.2.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2065,31 +2077,29 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CVE-2020-5194</t>
-        </is>
-      </c>
-      <c r="B36" s="1" t="n">
-        <v>43844</v>
+          <t>CVE-2006-6366</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2006-12-07</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>The zip API endpoint in Cerberus FTP Server 8 allows an authenticated attacker without zip permission to use the zip functionality via an unrestricted API endpoint. Improper permission verification occurs when calling the file/ajax_download_zip/zip_name endpoint. The result is that a user without permissions can zip and download files even if they do not have permission to view whether the file exists.</t>
+          <t>Cross-site scripting (XSS) vulnerability in includes/elements/spellcheck/spellwin.php in Cerberus Helpdesk 0.97.3, 2.0 through 2.7, 3.2.1, and 3.3 allows remote attackers to inject arbitrary web script or HTML via the js parameter.  NOTE: The provenance of this information is unknown; the details are obtained solely from third party information.</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5.4</v>
+        <v>6.8</v>
       </c>
       <c r="E36" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>CWE-639</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:8.0:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:helpdesk:0.97.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.6.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:2.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.2.317:*:*:*:*:*:*:*|cpe:2.3:a:cerberus:helpdesk:3.3:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2113,31 +2123,33 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CVE-2020-5196</t>
-        </is>
-      </c>
-      <c r="B37" s="1" t="n">
-        <v>43844</v>
+          <t>CVE-2008-6440</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2009-03-06</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cerberus FTP Server Enterprise Edition prior to versions 11.0.3 and 10.0.18 allows an authenticated attacker to create files, display hidden files, list directories, and list files without the permission to zip and download (or unzip and upload) files. There are multiple ways to bypass certain permissions by utilizing the zip and unzip features. As a result, users without permission can see files, folders, and hidden files, and can create directories without permission.</t>
+          <t>Cerberus Helpdesk before 4.0 (Build 600) allows remote attackers to obtain sensitive information via direct requests for "controllers ... that aren't standard helpdesk pages," possibly involving the (1) /display and (2) /kb URIs.</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8.1</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CWE-276</t>
+          <t>CWE-287</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
+          <t>cpe:2.3:a:cerberus:cerberus_helpdesk:2.5:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:*:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:0.97.3:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.0:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.1:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.2:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.3:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.4:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.6.1:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.7:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.7.1:development_release:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:2.649:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:3.2:*:*:*:*:*:*:*|cpe:2.3:a:webgroupmedia:cerberus_helpdesk:3.2.1:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2161,22 +2173,24 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CVE-2020-5195</t>
-        </is>
-      </c>
-      <c r="B38" s="1" t="n">
-        <v>43843</v>
+          <t>CVE-2012-6339</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2012-12-31</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Reflected XSS through an IMG element in Cerberus FTP Server prior to versions 11.0.1 and 10.0.17 allows a remote attacker to execute arbitrary JavaScript or HTML via a crafted public folder URL. This occurs because of the folder_up.png IMG element not properly sanitizing user-inserted directory paths. The path modification must be done on a publicly shared folder for a remote attacker to insert arbitrary JavaScript or HTML. The vulnerability impacts anyone who clicks the malicious link crafted by the attacker.</t>
+          <t>Multiple cross-site scripting (XSS) vulnerabilities in the administrative web interface in Cerberus FTP Server before 5.0.6.0 allow (1) remote attackers to inject arbitrary web script or HTML via a log entry that is not properly handled within the Log Manager component, and might allow (2) remote authenticated administrators to inject arbitrary web script or HTML via a Messages field to the servermanager program.</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>6.1</v>
+        <v>4.3</v>
       </c>
       <c r="E38" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2185,7 +2199,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.10.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.11.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.5.0:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2209,42 +2223,44 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CVE-2021-46778</t>
-        </is>
-      </c>
-      <c r="B39" s="1" t="n">
-        <v>44783</v>
+          <t>CVE-2013-4860</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2014-06-05</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Execution unit scheduler contention may lead to a side channel vulnerability found on AMD CPU microarchitectures codenamed “Zen 1”, “Zen 2” and “Zen 3” that use simultaneous multithreading (SMT). By measuring the contention level on scheduler queues an attacker may potentially leak sensitive information.</t>
+          <t>Radio Thermostat CT80 And CT50 with firmware 1.4.64 and earlier does not restrict access to the API, which allows remote attackers to change the operation mode, wifi connection settings, temperature thresholds, and other settings via unspecified vectors.</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E39" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CWE-203</t>
+          <t>CWE-264</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:amd:athlon_3050ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:athlon_3050ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:athlon_3150g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:athlon_3150g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:athlon_3150ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:athlon_3150ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7001_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7001:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7002_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7002:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7003_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7003:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7232p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7232p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7251_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7251:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7252_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7252:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7261_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7261:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7262_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7262:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7272_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7272:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7281_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7281:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7282_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7282:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_72f3_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_72f3:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7301_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7301:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7302_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7302:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7302p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7302p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7313_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7313:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7313p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7313p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7343_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7343:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7351_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7351:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7351p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7351p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7352_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7352:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7371_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7371:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7373x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7373x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_73f3_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_73f3:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7401_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7401:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7401p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7401p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7402_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7402:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7402p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7402p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7413_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7413:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7443_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7443:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7443p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7443p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7451_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7451:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7452_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7452:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7453_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7453:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7473x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7473x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_74f3_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_74f3:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7501_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7501:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7502_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7502:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7502p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7502p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7513_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7513:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7532_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7532:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7542_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7542:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7543_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7543:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7543p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7543p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7551_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7551:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7551p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7551p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7552_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7552:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7573x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7573x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_75f3_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_75f3:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7601_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7601:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7642_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7642:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7643_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7643:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7662_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7662:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7663_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7663:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7702_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7702:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7702p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7702p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7713_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7713:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7713p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7713p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7742_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7742:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7763_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7763:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7773x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7773x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f32_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f32:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f52_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f52:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f72_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f72:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7h12_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7h12:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_2200u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_2200u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_2300u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_2300u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3100_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3100:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3200u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3200u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3250u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3250u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3300g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3300g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3300u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3300u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3300x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3300x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3350u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3350u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3450u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3450u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3500c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3500c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3550h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3550h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3580u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3580u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3700c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3700c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3750h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3750h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3780u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3780u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_4300g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_4300g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_4300ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_4300ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_4300u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_4300u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5125c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5125c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5300g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5300g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5300ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5300ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5300u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5300u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5400u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5400u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5425c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5425c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5425u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5425u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_2500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_2500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_2600_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_2600:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_2600h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_2600h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_2600x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_2600x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_2700x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_2700x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3400g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3400g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3450g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3450g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3550h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3550h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3580u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3580u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600xt_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600xt:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5560u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5560u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600hs_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600hs:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5600x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5600x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5625c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5625c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5625u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5625u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5700g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5700g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5700ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5700ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_2700_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_2700:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_2700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_2700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_2700x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_2700x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_2800h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_2800h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3700x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3700x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3750h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3750h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3780u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3780u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3800x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3800x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3800xt_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3800xt:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4700g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4700g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4700ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4700ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4800h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4800h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4800u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4800u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5700g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5700g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5700ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5700ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5700x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5700x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5800h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5800h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5800hs_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5800hs:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5800u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5800u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5800x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5800x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5800x3d_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5800x3d:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5825c_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5825c:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5825u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5825u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3900x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3900x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3950x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3950x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_4900h_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_4900h:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_4900hs_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_4900hs:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5900hs_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5900hs:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5900hx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5900hx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5900x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5900x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5950x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5950x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5980hs_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5980hs:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_5980hx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_5980hx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_2920x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_2920x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_2950x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_2950x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_2970wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_2970wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_2990wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_2990wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3960x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3960x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3970x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3970x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3990x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3990x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3795wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3795wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3945wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3945wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3955wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3955wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3975wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3975wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3995wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3995wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_5945wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_5945wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_5955wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_5955wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_5965wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_5965wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_5975wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_5975wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_5995wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_5995wx:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:radiothermostat:ct50_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct50:-:*:*:*:*:*:*:*|cpe:2.3:o:radiothermostat:ct80_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:radiothermostat:ct80:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -2257,31 +2273,33 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CVE-2021-21877</t>
-        </is>
-      </c>
-      <c r="B40" s="1" t="n">
-        <v>44552</v>
+          <t>CVE-2015-3201</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2015-06-08</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Specially-crafted HTTP requests can lead to arbitrary command execution in “GET” requests. An attacker can make authenticated HTTP requests to trigger this vulnerability.</t>
+          <t>Thermostat before 2.0.0 uses world-readable permissions for the web.xml configuration file, which allows local users to obtain user credentials by reading the file.</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9.1</v>
+        <v>2.1</v>
       </c>
       <c r="E40" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CWE-78</t>
+          <t>CWE-200</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:lantronix:premierwave_2050_firmware:8.9.0.0:r4:*:*:*:*:*:*|cpe:2.3:h:lantronix:premierwave_2050:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:redhat:thermostat:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2305,179 +2323,147 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CVE-2021-37181</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="n">
-        <v>44453</v>
+          <t>CVE-2016-0870</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2016-09-19</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A vulnerability has been identified in Cerberus DMS V4.0 (All versions), Cerberus DMS V4.1 (All versions), Cerberus DMS V4.2 (All versions), Cerberus DMS V5.0 (All versions &lt; v5.0 QU1), Desigo CC Compact V4.0 (All versions), Desigo CC Compact V4.1 (All versions), Desigo CC Compact V4.2 (All versions), Desigo CC Compact V5.0 (All versions &lt; V5.0 QU1), Desigo CC V4.0 (All versions), Desigo CC V4.1 (All versions), Desigo CC V4.2 (All versions), Desigo CC V5.0 (All versions &lt; V5.0 QU1). The application deserialises untrusted data without sufficient validations, that could result in an arbitrary deserialization. This could allow an unauthenticated attacker to execute code in the affected system. The CCOM communication component used for Windows App / Click-Once and IE Web / XBAP client connectivity are affected by the vulnerability.</t>
+          <t>The web server in Trane Tracer SC 4.2.1134 and earlier allows remote attackers to read sensitive configuration files via a direct request.</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>10</v>
+        <v>5.3</v>
       </c>
       <c r="E41" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>CWE-502</t>
+          <t>CWE-200</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:siemens:cerberus_dms:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_dms:5.0:-:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:5.0:-:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.0:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.1:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:4.2:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:5.0:-:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Maybe</t>
-        </is>
-      </c>
+          <t>cpe:2.3:a:trane:tracer_sc:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Siemens Cerberus DMS and Desigo CC are enterprise building management/fire alarm platforms used in commercial buildings, not residential homes. Fails criterion 1 — not a residential deployment without dedicated security oversight.</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CVE-2021-27952</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="n">
-        <v>44411</v>
+          <t>CVE-2016-4526</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2016-09-19</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hardcoded default root credentials exist on the ecobee3 lite 4.5.81.200 device. This allows a threat actor to gain access to the password-protected bootloader environment through the serial console.</t>
+          <t>ABB DataManagerPro 1.x before 1.7.1 allows local users to gain privileges by replacing a DLL file in the package directory.</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="E42" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>CWE-798</t>
+          <t>CWE-427</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>cpe:2.3:a:trane:tracer_sc:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CVE-2021-27953</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="n">
-        <v>44411</v>
+          <t>CVE-2018-10122</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2018-04-16</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>A NULL pointer dereference vulnerability exists on the ecobee3 lite 4.5.81.200 device in the HomeKit Wireless Access Control setup process. A threat actor can exploit this vulnerability to cause a denial of service, forcing the device to reboot via a crafted HTTP request.</t>
+          <t>QingDao Nature Easy Soft Chanzhi Enterprise Portal System (aka chanzhieps) pro1.6 allows remote attackers to read arbitrary files via directory traversal sequences in the pathname parameter to www/file.php.</t>
         </is>
       </c>
       <c r="D43" t="n">
         <v>7.5</v>
       </c>
       <c r="E43" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>CWE-476</t>
+          <t>CWE-22</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>cpe:2.3:a:chanzhi:chanzhi:pro1.6:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CVE-2021-27954</t>
-        </is>
-      </c>
-      <c r="B44" s="1" t="n">
-        <v>44411</v>
+          <t>CVE-2018-6402</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2020-04-14</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>A heap-based buffer overflow vulnerability exists on the ecobee3 lite 4.5.81.200 device in the HKProcessConfig function of the HomeKit Wireless Access Control setup process. A threat actor can exploit this vulnerability to force the device to connect to a SSID or cause a denial of service.</t>
+          <t>Ecobee Ecobee4 4.2.0.171 devices can be forced to deauthenticate and connect to an unencrypted Wi-Fi network with the same SSID, even if the device settings specify use of encryption such as WPA2, as long as the competing network has a stronger signal. An attacker must be able to set up a nearby SSID, similar to an "Evil Twin" attack.</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8.199999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="E44" t="n">
         <v>3.1</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>CWE-787</t>
+          <t>CWE-327</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:ecobee:ecobee4_firmware:4.2.0.171:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee4:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2501,31 +2487,33 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CVE-2022-43704</t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>44946</v>
+          <t>CVE-2021-27952</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2021-08-03</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The Sinilink XY-WFT1 WiFi Remote Thermostat, running firmware 1.3.6, allows an attacker to bypass the intended requirement to communicate using MQTT. It is possible to replay Sinilink aka SINILINK521 protocol (udp/1024) commands interfacing directly with the target device. This, in turn, allows for an attack to control the onboard relay without requiring authentication via the mobile application. This might result in an unacceptable temperature within the target device's physical environment.</t>
+          <t>Hardcoded default root credentials exist on the ecobee3 lite 4.5.81.200 device. This allows a threat actor to gain access to the password-protected bootloader environment through the serial console.</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E45" t="n">
         <v>3.1</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CWE-294</t>
+          <t>CWE-798</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:sinilink:xy-wft1_firmware:1.3.6:*:*:*:*:*:*:*|cpe:2.3:h:sinilink:xy-wft1:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2549,88 +2537,88 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CVE-2022-33139</t>
-        </is>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>44733</v>
+          <t>CVE-2021-27953</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2021-08-03</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>A vulnerability has been identified in Cerberus DMS (All versions), Desigo CC (All versions), Desigo CC Compact (All versions), SIMATIC WinCC OA V3.16 (All versions in default configuration), SIMATIC WinCC OA V3.17 (All versions in non-default configuration), SIMATIC WinCC OA V3.18 (All versions in non-default configuration). Affected applications use client-side only authentication, when neither server-side authentication (SSA) nor Kerberos authentication is enabled. In this configuration, attackers could impersonate other users or exploit the client-server protocol without being authenticated.</t>
+          <t>A NULL pointer dereference vulnerability exists on the ecobee3 lite 4.5.81.200 device in the HomeKit Wireless Access Control setup process. A threat actor can exploit this vulnerability to cause a denial of service, forcing the device to reboot via a crafted HTTP request.</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="E46" t="n">
         <v>3.1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>CWE-603|CWE-287</t>
+          <t>CWE-476</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:siemens:cerberus_dms:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:desigo_cc_compact:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.16:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.17:*:*:*:*:*:*:*|cpe:2.3:a:siemens:wincc_open_architecture:3.18:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Siemens Cerberus DMS and WinCC OA are industrial SCADA/building automation platforms. Same reasoning as CVE-2021-37181 — fails criterion 1 (residential deployment without dedicated security oversight).</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CVE-2023-46892</t>
-        </is>
-      </c>
-      <c r="B47" s="1" t="n">
-        <v>45314</v>
+          <t>CVE-2021-27954</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2021-08-03</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>The radio frequency communication protocol being used by Meross MSH30Q 4.5.23 is vulnerable to replay attacks, allowing attackers to record and replay previously captured communication to execute unauthorized commands or actions (e.g., thermostat's temperature).</t>
+          <t>A heap-based buffer overflow vulnerability exists on the ecobee3 lite 4.5.81.200 device in the HKProcessConfig function of the HomeKit Wireless Access Control setup process. A threat actor can exploit this vulnerability to force the device to connect to a SSID or cause a denial of service.</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>8.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E47" t="n">
         <v>3.1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>CWE-294</t>
+          <t>CWE-787</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:meross:msh30q_firmware:4.5.23:*:*:*:*:*:*:*|cpe:2.3:h:meross:msh30q:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:ecobee:ecobee3_lite_firmware:4.5.81.200:*:*:*:*:*:*:*|cpe:2.3:h:ecobee:ecobee3_lite:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2649,31 +2637,33 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CVE-2023-30962</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="n">
-        <v>45181</v>
+          <t>CVE-2019-25046</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2021-06-10</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>The Gotham Cerberus service was found to have a stored cross-site scripting (XSS) vulnerability that could have allowed an attacker with access to Gotham to launch attacks against other users. This vulnerability is resolved in Cerberus 100.230704.0-27-g031dd58 .</t>
+          <t>The Web Client in Cerberus FTP Server Enterprise before 10.0.19 and 11.x before 11.0.4 allows XSS via an SVG document.</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="E48" t="n">
         <v>3.1</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>CWE-434|CWE-79</t>
+          <t>CWE-79</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:palantir:gotham_cerberus:*:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:enterprise:*:*:*</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2697,92 +2687,84 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>CVE-2021-38448</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2021-11-22</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The affected controllers do not properly sanitize the input containing code syntax. As a result, an attacker could craft code to alter the intended controller flow of the software.</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>CWE-94</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:trane:symbio_700:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:odyssey_split_systems:-:*:*:*:*:*:*:*|cpe:2.3:a:trane:symbio_800:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:intellipak_1:-:*:*:*:*:*:*:*|cpe:2.3:h:trane:intellipak_2:-:*:*:*:*:*:*:*|cpe:2.3:h:trane:ascend_air-cooled_chiller_acr:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>CVE-2023-4212</t>
         </is>
       </c>
-      <c r="B49" s="1" t="n">
-        <v>45160</v>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2023-08-22</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
         <is>
           <t xml:space="preserve">
 ​A command injection vulnerability exists in Trane XL824, XL850, XL1050, and Pivot thermostats allowing an attacker to execute arbitrary commands as root using a specially crafted filename. The vulnerability requires physical access to the device via a USB stick.
 </t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D50" t="n">
         <v>6.8</v>
-      </c>
-      <c r="E49" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>CWE-74|CWE-77</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>cpe:2.3:o:trane:xl824_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl824:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:xl850_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl850:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:xl1050_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl1050:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:pivot_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:pivot:-:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>CVE-2023-20593</t>
-        </is>
-      </c>
-      <c r="B50" s="1" t="n">
-        <v>45131</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>An issue in “Zen 2” CPUs, under specific microarchitectural circumstances, may allow an attacker to potentially access sensitive information.</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>5.5</v>
       </c>
       <c r="E50" t="n">
         <v>3.1</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>CWE-209</t>
+          <t>CWE-74|CWE-77</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:xen:xen:4.14.0:*:*:*:*:*:x86:*|cpe:2.3:o:xen:xen:4.15.0:*:*:*:*:*:x86:*|cpe:2.3:o:xen:xen:4.16.0:*:*:*:*:*:x86:*|cpe:2.3:o:xen:xen:4.17.0:*:*:*:*:*:x86:*|cpe:2.3:o:debian:debian_linux:10.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:11.0:*:*:*:*:*:*:*|cpe:2.3:o:debian:debian_linux:12.0:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3100_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3100:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_3300x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_3300x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3500_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3500:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3500x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3500x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_3600xt_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_3600xt:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3700x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3700x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3800x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3800x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_3800xt_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_3800xt:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3900_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3900:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3900x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3900x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3900xt_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3900xt:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_3950x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_3950x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_9_pro_3900_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_9_pro_3900:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3995wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3995wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3975wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3975wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3955wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3955wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_pro_3945wx_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_pro_3945wx:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3990x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3990x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3970x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3970x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_threadripper_3960x_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_threadripper_3960x:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4700g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4700g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_4700ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_4700ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_4600ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_4600ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_4300g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_4300g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_4300ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_4300ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_pro_4450u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_pro_4450u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_pro_4350ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_pro_4350ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_pro_4350g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_pro_4350g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_pro_4200g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_pro_4200g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_pro_4650ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_pro_4650ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_pro_4650g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_pro_4650g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_pro_4400g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_pro_4400g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_pro_4750u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_pro_4750u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_pro_4750ge_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_pro_4750ge:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_pro_4750g_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_pro_4750g:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_7_5700u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_7_5700u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_5500u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_5500u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_5300u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_5300u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_5_7520u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_5_7520u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:ryzen_3_7320u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:ryzen_3_7320u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:athlon_gold_7220u_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:athlon_gold_7220u:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7232p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7232p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7302p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7302p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7402p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7402p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7502p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7502p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7702p_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7702p:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7252_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7252:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7262_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7262:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7272_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7272:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7282_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7282:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7302_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7302:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7352_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7352:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7402_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7402:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7452_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7452:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7502_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7502:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7532_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7532:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7542_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7542:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7552_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7552:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7642_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7642:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7662_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7662:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7702_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7702:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7742_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7742:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7h12_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7h12:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f32_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f32:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f52_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f52:-:*:*:*:*:*:*:*|cpe:2.3:o:amd:epyc_7f72_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:amd:epyc_7f72:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:o:trane:xl824_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl824:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:xl850_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl850:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:xl1050_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:xl1050:-:*:*:*:*:*:*:*|cpe:2.3:o:trane:pivot_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:pivot:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -2795,38 +2777,44 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CVE-2023-24678</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="n">
-        <v>45002</v>
+          <t>CVE-2023-30962</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2023-09-12</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>A vulnerability in Centralite Pearl Thermostat 0x04075010 allows attackers to cause a Denial of Service (DoS) via a crafted Zigbee message.</t>
+          <t>The Gotham Cerberus service was found to have a stored cross-site scripting (XSS) vulnerability that could have allowed an attacker with access to Gotham to launch attacks against other users. This vulnerability is resolved in Cerberus 100.230704.0-27-g031dd58 .</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>7.5</v>
+        <v>5.4</v>
       </c>
       <c r="E51" t="n">
         <v>3.1</v>
       </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>CWE-434|CWE-79</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:centralite:pearl_firmware:0x04075010:*:*:*:*:*:*:*|cpe:2.3:h:centralite:pearl:-:*:*:*:*:*:*:*</t>
+          <t>cpe:2.3:a:palantir:gotham_cerberus:*:*:*:*:*:*:*:*</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -2839,91 +2827,82 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CVE-2024-42642</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="n">
-        <v>45539</v>
+          <t>CVE-2023-6339</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2024-01-02</t>
+        </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Micron Crucial MX500 Series Solid State Drives M3CR046 is vulnerable to Buffer Overflow, which can be triggered by sending specially crafted ATA packets from the host to the drive controller. NOTE: The supplier states that this vulnerability was fully remediated in December 2024 and that updated firmware is available through Crucial’s official support page.</t>
+          <t>Google Nest WiFi Pro root code-execution &amp; user-data compromise</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E52" t="n">
         <v>3.1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>CWE-787|CWE-120</t>
+          <t>CWE-311</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>cpe:2.3:o:crucial:mx500_firmware:m3cr046:*:*:*:*:*:*:*|cpe:2.3:h:crucial:ct1000mx500ssd1:-:*:*:*:*:*:*:*|cpe:2.3:h:crucial:ct2000mx500ssd1:-:*:*:*:*:*:*:*|cpe:2.3:h:crucial:ct250mx500ssd1:-:*:*:*:*:*:*:*|cpe:2.3:h:crucial:ct4000mx500ssd1:-:*:*:*:*:*:*:*|cpe:2.3:h:crucial:ct500mx500ssd1:-:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:google:nest_wifi_pro_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:google:nest_wifi_pro:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CVE-2024-0397</t>
-        </is>
-      </c>
-      <c r="B53" s="1" t="n">
-        <v>45460</v>
+          <t>CVE-2023-46892</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2024-01-23</t>
+        </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A defect was discovered in the Python “ssl” module where there is a memory
-race condition with the ssl.SSLContext methods “cert_store_stats()” and
-“get_ca_certs()”. The race condition can be triggered if the methods are
-called at the same time as certificates are loaded into the SSLContext,
-such as during the TLS handshake with a certificate directory configured.
-This issue is fixed in CPython 3.10.14, 3.11.9, 3.12.3, and 3.13.0a5.</t>
+          <t>The radio frequency communication protocol being used by Meross MSH30Q 4.5.23 is vulnerable to replay attacks, allowing attackers to record and replay previously captured communication to execute unauthorized commands or actions (e.g., thermostat's temperature).</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>7.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E53" t="n">
         <v>3.1</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>CWE-362</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
+          <t>CWE-294</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>cpe:2.3:o:meross:msh30q_firmware:4.5.23:*:*:*:*:*:*:*|cpe:2.3:h:meross:msh30q:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
@@ -2936,122 +2915,138 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CVE-2024-5052</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="n">
-        <v>45429</v>
+          <t>CVE-2024-22039</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Denial of Service (DoS) vulnerability for Cerberus Enterprise 8.0.10.3 web administration. The vulnerability exists when the web server, default port 10001, attempts to process a large number of incomplete HTTP requests.</t>
+          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions &lt; IP8), Cerberus PRO EN Fire Panel FC72x IP6 (All versions &lt; IP6 SR3), Cerberus PRO EN Fire Panel FC72x IP7 (All versions &lt; IP7 SR5), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions &lt; V3.0.6602), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.0.5016), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions &lt; V3.2.6601), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.2.5015), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions &lt; MP8), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions &lt; MP6 SR3), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions &lt; MP7 SR5), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions &lt; V3.0.6602), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.0.5016), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions &lt; V3.2.6601), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.2.5015), Sinteso Mobile (All versions &lt; V3.0.0). The network communication library in affected systems does not validate the length of certain X.509 certificate attributes which might result in a stack-based buffer overflow.
+This could allow an unauthenticated remote attacker to execute code on the underlying operating system with root privileges.</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E54" t="n">
         <v>3.1</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>CWE-400</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
+          <t>CWE-120</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:siemens:cerberus_pro_en_engineering_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_fire_panel_fc72x:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_x200_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_x300_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_engineering_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_fire_panel_fc20:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_x200_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_x300_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_mobile:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Siemens Cerberus PRO EN is a professional fire detection system primarily deployed in commercial buildings. Residential fire panels do exist but this is an enterprise-grade product line. CPE confirms Siemens commercial product — not typical home IoT.</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CVE-2024-1630</t>
-        </is>
-      </c>
-      <c r="B55" s="1" t="n">
-        <v>45426</v>
+          <t>CVE-2024-22040</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Path traversal vulnerability in “getAllFolderContents” function of Common Service Desktop, a GE HealthCare ultrasound device component</t>
+          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions), Cerberus PRO EN Fire Panel FC72x IP6 (All versions), Cerberus PRO EN Fire Panel FC72x IP7 (All versions), Cerberus PRO EN Fire Panel FC72x IP8 (All versions &lt; IP8 SR4), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.3.5618), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.3.5617), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions), Sinteso FS20 EN Fire Panel FC20 MP8 (All versions &lt; MP8 SR4), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.3.5618), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.3.5617), Sinteso Mobile (All versions). The network communication library in affected systems insufficiently validates HMAC values which might result in a buffer overread.
+This could allow an unauthenticated remote attacker to crash the network service.</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="E55" t="n">
         <v>3.1</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>CWE-22</t>
+          <t>CWE-125</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr"/>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Same as CVE-2024-22039 — Siemens Cerberus PRO EN commercial fire detection system. No CPE string available to further confirm device context.</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CVE-2024-22039</t>
-        </is>
-      </c>
-      <c r="B56" s="1" t="n">
-        <v>45363</v>
+          <t>CVE-2024-22041</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions &lt; IP8), Cerberus PRO EN Fire Panel FC72x IP6 (All versions &lt; IP6 SR3), Cerberus PRO EN Fire Panel FC72x IP7 (All versions &lt; IP7 SR5), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions &lt; V3.0.6602), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.0.5016), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions &lt; V3.2.6601), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.2.5015), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions &lt; MP8), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions &lt; MP6 SR3), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions &lt; MP7 SR5), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions &lt; V3.0.6602), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.0.5016), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions &lt; V3.2.6601), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.2.5015), Sinteso Mobile (All versions &lt; V3.0.0). The network communication library in affected systems does not validate the length of certain X.509 certificate attributes which might result in a stack-based buffer overflow.
-This could allow an unauthenticated remote attacker to execute code on the underlying operating system with root privileges.</t>
+          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions), Cerberus PRO EN Fire Panel FC72x IP6 (All versions), Cerberus PRO EN Fire Panel FC72x IP7 (All versions), Cerberus PRO EN Fire Panel FC72x IP8 (All versions &lt; IP8 SR4), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.3.5618), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.3.5617), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions), Sinteso FS20 EN Fire Panel FC20 MP8 (All versions &lt; MP8 SR4), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.3.5618), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.3.5617), Sinteso Mobile (All versions). The network communication library in affected systems improperly handles memory buffers when parsing X.509 certificates.
+This could allow an unauthenticated remote attacker to crash the network service.</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>9.800000000000001</v>
+        <v>7.5</v>
       </c>
       <c r="E56" t="n">
         <v>3.1</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CWE-120</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>cpe:2.3:a:siemens:cerberus_pro_en_engineering_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_fire_panel_fc72x:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_x200_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:cerberus_pro_en_x300_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_engineering_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_fire_panel_fc20:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_x200_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_fs20_en_x300_cloud_distribution:*:*:*:*:*:*:*:*|cpe:2.3:a:siemens:sinteso_mobile:*:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
+          <t>CWE-119</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3065,7 +3060,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Siemens Cerberus PRO EN is a professional fire detection system primarily deployed in commercial buildings. Residential fire panels do exist but this is an enterprise-grade product line. CPE confirms Siemens commercial product — not typical home IoT.</t>
+          <t>Same as CVE-2024-22039 — Siemens Cerberus PRO EN commercial fire detection system. No CPE string available.</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -3077,16 +3072,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CVE-2024-22040</t>
-        </is>
-      </c>
-      <c r="B57" s="1" t="n">
-        <v>45363</v>
+          <t>CVE-2024-5052</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2024-05-17</t>
+        </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions), Cerberus PRO EN Fire Panel FC72x IP6 (All versions), Cerberus PRO EN Fire Panel FC72x IP7 (All versions), Cerberus PRO EN Fire Panel FC72x IP8 (All versions &lt; IP8 SR4), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.3.5618), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.3.5617), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions), Sinteso FS20 EN Fire Panel FC20 MP8 (All versions &lt; MP8 SR4), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.3.5618), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.3.5617), Sinteso Mobile (All versions). The network communication library in affected systems insufficiently validates HMAC values which might result in a buffer overread.
-This could allow an unauthenticated remote attacker to crash the network service.</t>
+          <t>Denial of Service (DoS) vulnerability for Cerberus Enterprise 8.0.10.3 web administration. The vulnerability exists when the web server, default port 10001, attempts to process a large number of incomplete HTTP requests.</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3097,111 +3093,102 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>CWE-125</t>
+          <t>CWE-400</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Maybe</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Same as CVE-2024-22039 — Siemens Cerberus PRO EN commercial fire detection system. No CPE string available to further confirm device context.</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CVE-2024-22041</t>
-        </is>
-      </c>
-      <c r="B58" s="1" t="n">
-        <v>45363</v>
+          <t>CVE-2025-6260</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2025-07-24</t>
+        </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>A vulnerability has been identified in Cerberus PRO EN Engineering Tool (All versions), Cerberus PRO EN Fire Panel FC72x IP6 (All versions), Cerberus PRO EN Fire Panel FC72x IP7 (All versions), Cerberus PRO EN Fire Panel FC72x IP8 (All versions &lt; IP8 SR4), Cerberus PRO EN X200 Cloud Distribution IP7 (All versions), Cerberus PRO EN X200 Cloud Distribution IP8 (All versions &lt; V4.3.5618), Cerberus PRO EN X300 Cloud Distribution IP7 (All versions), Cerberus PRO EN X300 Cloud Distribution IP8 (All versions &lt; V4.3.5617), Cerberus PRO UL Compact Panel FC922/924 (All versions &lt; MP4), Cerberus PRO UL Engineering Tool (All versions &lt; MP4), Cerberus PRO UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Desigo Fire Safety UL Compact Panel FC2025/2050 (All versions &lt; MP4), Desigo Fire Safety UL Engineering Tool (All versions &lt; MP4), Desigo Fire Safety UL X300 Cloud Distribution (All versions &lt; V4.3.0001), Sinteso FS20 EN Engineering Tool (All versions), Sinteso FS20 EN Fire Panel FC20 MP6 (All versions), Sinteso FS20 EN Fire Panel FC20 MP7 (All versions), Sinteso FS20 EN Fire Panel FC20 MP8 (All versions &lt; MP8 SR4), Sinteso FS20 EN X200 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X200 Cloud Distribution MP8 (All versions &lt; V4.3.5618), Sinteso FS20 EN X300 Cloud Distribution MP7 (All versions), Sinteso FS20 EN X300 Cloud Distribution MP8 (All versions &lt; V4.3.5617), Sinteso Mobile (All versions). The network communication library in affected systems improperly handles memory buffers when parsing X.509 certificates.
-This could allow an unauthenticated remote attacker to crash the network service.</t>
+          <t>The embedded web server on the thermostat listed version ranges contain a vulnerability that allows unauthenticated attackers, either on the local area network or from the Internet via a router with port forwarding set up, to gain direct access to the thermostat's embedded web server and reset user credentials by manipulating specific elements of the embedded web interface.</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E58" t="n">
         <v>3.1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>CWE-119</t>
+          <t>CWE-306</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Maybe</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Maybe</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Same as CVE-2024-22039 — Siemens Cerberus PRO EN commercial fire detection system. No CPE string available.</t>
-        </is>
-      </c>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CVE-2025-67124</t>
-        </is>
-      </c>
-      <c r="B59" s="1" t="n">
-        <v>46045</v>
+          <t>CVE-2025-7718</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>A TOCTOU and symlink race in svenstaro/miniserve 0.32.0 upload finalization (when uploads are enabled) can allow an attacker to overwrite arbitrary files outside the intended upload/document root in deployments where the attacker can create/replace filesystem entries in the upload destination directory (e.g., shared writable directory/volume).</t>
+          <t>The Resideo Plugin for Resideo - Real Estate WordPress Theme plugin for WordPress is vulnerable to privilege escalation via account takeover in all versions up to, and including, 2.5.4. This is due to the plugin not properly validating a user's identity prior to updating their details like email. This makes it possible for authenticated attackers, with Subscriber-level access and above, to change arbitrary user's email addresses, including administrators, and leverage that to reset the user's password and gain access to their account.</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>6.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E59" t="n">
         <v>3.1</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>CWE-59|CWE-367</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>cpe:2.3:a:svenstaro:miniserve:0.32.0:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
+          <t>CWE-639</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>No</t>
@@ -3223,59 +3210,51 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CVE-2025-7718</t>
-        </is>
-      </c>
-      <c r="B60" s="1" t="n">
-        <v>45910</v>
+          <t>CVE-2022-50918</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Resideo Plugin for Resideo - Real Estate WordPress Theme plugin for WordPress is vulnerable to privilege escalation via account takeover in all versions up to, and including, 2.5.4. This is due to the plugin not properly validating a user's identity prior to updating their details like email. This makes it possible for authenticated attackers, with Subscriber-level access and above, to change arbitrary user's email addresses, including administrators, and leverage that to reset the user's password and gain access to their account.</t>
+          <t>VIVE Runtime Service 1.0.0.4 contains an unquoted service path vulnerability that allows local users to execute arbitrary code with elevated system privileges. Attackers can exploit the unquoted binary path by placing malicious executables in specific system directories to gain LocalSystem access during service startup.</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>8.800000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="E60" t="n">
         <v>3.1</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CWE-639</t>
+          <t>CWE-428</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CVE-2025-6260</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="n">
-        <v>45862</v>
+          <t>CVE-2026-28252</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>The embedded web server on the thermostat listed version ranges contain a vulnerability that allows unauthenticated attackers, either on the local area network or from the Internet via a router with port forwarding set up, to gain direct access to the thermostat's embedded web server and reset user credentials by manipulating specific elements of the embedded web interface.</t>
+          <t>A Use of a Broken or Risky Cryptographic Algorithm vulnerability in Trane Tracer SC, Tracer SC+, and Tracer Concierge could allow an attacker to bypass authentication and gain root-level access to the device.</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3286,71 +3265,477 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CWE-306</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Maybe</t>
-        </is>
-      </c>
+          <t>CWE-327</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack1:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack2:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack3:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack4:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack5:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack6:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="L61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CVE-2026-23634</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="n">
-        <v>46038</v>
+          <t>CVE-2026-28253</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Pepr is a type safe K8s middleware. Prior to 1.0.5 , Pepr defaults to a cluster-admin RBAC configuration and does not explicitly force or enforce least-privilege guidance for module authors. The default behavior exists to make the “getting started” experience smooth: new users can experiment with Pepr and create resources dynamically without needing to pre-configure RBAC. This vulnerability is fixed in 1.0.5.</t>
+          <t>A Memory Allocation with Excessive Size Value vulnerability in Trane Tracer SC, Tracer SC+, and Tracer Concierge could allow an unauthenticated attacker to cause a denial-of-service condition</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>4.3</v>
+        <v>7.5</v>
       </c>
       <c r="E62" t="n">
         <v>3.1</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>CWE-272</t>
+          <t>CWE-789</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>cpe:2.3:a:defenseunicorns:pepr:*:*:*:*:*:*:*:*</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack1:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack2:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack3:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack4:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack5:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack6:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
+      <c r="L62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CVE-2026-28254</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>A Missing Authorization vulnerability in Trane Tracer SC, Tracer SC+, and Tracer Concierge could allow an unauthenticated attacker to access sensitive information through unprotected APIs.</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E63" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>CWE-862</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack1:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack2:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack3:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack4:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack5:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack6:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CVE-2026-28255</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>A Use of Hard-coded Credentials vulnerability in Trane Tracer SC, Tracer SC+, and Tracer Concierge could allow an attacker to disclose sensitive information and take over accounts.</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>CWE-798</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack1:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack2:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack3:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack4:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack5:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack6:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CVE-2026-28256</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>A Use of Hard-coded, Security-relevant Constants vulnerability in Trane Tracer SC, Tracer SC+, and Tracer Concierge could allow an attacker to disclose sensitive information and take over accounts.</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E65" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>CWE-547</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>cpe:2.3:o:trane:tracer_sc\+_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc\+:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack1:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack2:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack3:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack4:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack5:*:*:*:*:*:*|cpe:2.3:o:trane:tracer_sc_firmware:4.4:service_pack6:*:*:*:*:*:*|cpe:2.3:h:trane:tracer_sc:*:*:*:*:*:*:*:*|cpe:2.3:a:trane:tracer_concierge:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>CVE-2019-25708</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Heatmiser Wifi Thermostat 1.7 contains a cross-site request forgery vulnerability that allows attackers to change administrator credentials by tricking authenticated users into submitting malicious requests. Attackers can craft HTML forms targeting the networkSetup.htm endpoint with parameters usnm, usps, and cfps to modify the admin username and password without user consent.</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E66" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>CWE-352</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:heatmiser:wifi_thermostat:1.7:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>CVE-2026-6265</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Insecure preserved inherited permissions vulnerability in Cerberus FTP Server on Windows allows Privilege Escalation.This issue has been resolved in Cerberus FTP Server: 2026.1</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="E67" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>CWE-278</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>CVE-2018-25396</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Heatmiser Wifi Thermostat 1.7 contains a credential disclosure vulnerability that allows unauthenticated attackers to retrieve administrative credentials by accessing the networkSetup.htm page. Attackers can request the networkSetup.htm endpoint and extract plaintext username and password values from HTML form fields to gain administrative access to the thermostat.</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E68" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CWE-256</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>CVE-2008-3397</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2008-07-31</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Cross-site scripting (XSS) vulnerability in Runesoft Cerberus CMS before 3_1.4_0.9 allows remote attackers to inject arbitrary web script or HTML via a cerberus_user cookie.</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E69" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CWE-79</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:runesoft:cerberus_cms:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>CVE-2012-4006</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2012-08-17</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>The GREE application before 1.4.0, GREE Tanken Dorirando application before 1.0.7, GREE Tsurisuta application before 1.5.0, GREE Monpura application before 1.1.1, GREE Kaizokuoukoku Columbus application before 1.3.5, GREE haconiwa application before 1.1.0, GREE Seisen Cerberus application before 1.1.0, and KDDI&amp;GREE GREE Market application before 2.1.2 for Android do not properly implement the WebView class, which allows remote attackers to obtain sensitive information via a crafted application.</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>CWE-200</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:gree:gree:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:haconiwa:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:kaizokuoukoku_columbus:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:monpura:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:seisen_cerberus:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:tanken_dorirando:*:*:*:*:*:*:*:*|cpe:2.3:a:gree:tsurisuta:*:*:*:*:*:*:*:*|cpe:2.3:a:kddi_\&amp;_gree:gree_market:*:*:*:*:*:*:*:*|cpe:2.3:o:google:android:*:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>CVE-2012-2999</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2012-10-04</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Multiple cross-site request forgery (CSRF) vulnerabilities in the web interface in Cerberus FTP Server before 5.0.5.0 allow remote attackers to hijack the authentication of administrators for requests that (1) add a user account or (2) reconfigure the state of the FTP service, as demonstrated by a request to usermanager/users/modify.</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>CWE-352</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.4.2:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>CVE-2012-5301</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2012-10-04</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>The default configuration of Cerberus FTP Server before 5.0.4.0 supports the DES cipher for SSH sessions, which makes it easier for remote attackers to obtain sensitive information by sniffing the network and performing a brute-force attack on the encrypted data.</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>5</v>
+      </c>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>CWE-310</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>cpe:2.3:a:cerberusftp:ftp_server:*:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.0:-:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.03:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.05:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.6:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:1.71:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.0:beta4:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.01:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.02:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.2:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta1:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.4:beta3:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.11:beta2:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.15:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.16:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.21:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.22:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.23:beta:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.31:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.32:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.41:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.42:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.43:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.44:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.45:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.46:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.47:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.48:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.49:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:2.50:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.7.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:3.1.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.9:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.0.11:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.2.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.3.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.4.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.5.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.7.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.8.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.9.8:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.10.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:4.0.11.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.3:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.4:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.5:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.6:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.0.7:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.1:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.1.2:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.2.0:*:*:*:*:*:*:*|cpe:2.3:a:cerberusftp:ftp_server:5.0.3.0:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
         <is>
           <t>High</t>
         </is>

</xml_diff>